<commit_message>
fix(b6): comma-percent shared-parser fix + 18-state retro-verify + surgical deliverable re-import
Root cause (reframed from wrapped-name): row regexes rejected thousands-comma
percentages (1,830.500%) -> silent 0-row/partial/wrong-value extraction.
_FS_PCT comma-tolerant core + additive shapes H/I/J; test_b6_parser_shapes.py
41 PASS (AK native == recover_ak_cfpc adjudication; pre-B6 shapes byte-identical).
Full 5,113-PDF old-vs-new diff: 5,098 byte-identical, 15 adjudicated diffs.
Recovered: IL active Defend CFPC-134419708 (-4.38%/334k ph) + back-ext, WV
wrong-value 0->2.8%, GA rollups source-true, VT/NM/VA/WA 0% completeness.
Surgical apply preserves GA/NM AM-Best tier enrichment (append-only); all_states
2947->2963, mtime re-pinned 2026-06-11. B6 closed, B7 (Temp-purge) opened.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Insurance Rate Data Scraper/output/ga_final_rates.xlsx
+++ b/Insurance Rate Data Scraper/output/ga_final_rates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U481"/>
+  <dimension ref="A1:U486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,7 +622,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -723,7 +722,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -824,7 +822,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -925,7 +922,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1026,7 +1022,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1127,7 +1122,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1228,7 +1222,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1329,7 +1322,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1430,7 +1422,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1531,7 +1522,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1942,7 +1932,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4908,7 +4897,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5009,7 +4997,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5110,7 +5097,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5211,7 +5197,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5312,7 +5297,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5413,7 +5397,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5514,7 +5497,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5615,7 +5597,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5716,7 +5697,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5817,7 +5797,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6338,7 +6317,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6649,7 +6627,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6750,7 +6727,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -6851,7 +6827,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -6952,7 +6927,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7053,7 +7027,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7154,7 +7127,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7255,7 +7227,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7356,7 +7327,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7457,7 +7427,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7558,7 +7527,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7654,7 +7622,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7750,7 +7717,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -7846,7 +7812,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7947,7 +7912,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8048,7 +8012,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8149,7 +8112,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8250,7 +8212,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8351,7 +8312,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8452,7 +8412,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -8553,7 +8512,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -8654,7 +8612,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -8755,7 +8712,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -8856,7 +8812,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8957,7 +8912,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9583,7 +9537,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9684,7 +9637,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -9785,7 +9737,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10201,7 +10152,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10407,7 +10357,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -10508,7 +10457,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -10814,7 +10762,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -10910,7 +10857,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -11006,7 +10952,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -11102,7 +11047,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -11298,7 +11242,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -11394,7 +11337,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -11490,7 +11432,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -11586,7 +11527,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -11682,7 +11622,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -11778,7 +11717,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -11874,7 +11812,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -11970,7 +11907,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -12066,7 +12002,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -12162,7 +12097,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -12258,7 +12192,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -14059,7 +13992,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -14160,7 +14092,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -14261,7 +14192,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -14362,7 +14292,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -14778,7 +14707,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -14879,7 +14807,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -14980,7 +14907,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -15081,7 +15007,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -15182,7 +15107,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -15283,7 +15207,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -15384,7 +15307,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -15485,7 +15407,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -15586,7 +15507,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -15687,7 +15607,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -15998,7 +15917,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -16099,7 +16017,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -16190,7 +16107,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -16281,7 +16197,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -16372,7 +16287,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -16463,7 +16377,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -16554,7 +16467,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -16645,7 +16557,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -16736,7 +16647,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -16827,7 +16737,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -16918,7 +16827,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -17009,7 +16917,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -19000,7 +18907,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -19101,7 +19007,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -19202,7 +19107,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -19303,7 +19207,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -19404,7 +19307,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -19505,7 +19407,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -19606,7 +19507,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -19707,7 +19607,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -19808,7 +19707,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -19909,7 +19807,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -20010,7 +19907,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -20216,7 +20112,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -20317,7 +20212,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -20418,7 +20312,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -20519,7 +20412,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -20620,7 +20512,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -20721,7 +20612,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -20822,7 +20712,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -21028,7 +20917,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -21129,7 +21017,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -21545,7 +21432,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -21646,7 +21532,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -21747,7 +21632,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -21848,7 +21732,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -21949,7 +21832,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -22050,7 +21932,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -22151,7 +22032,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -22252,7 +22132,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -22353,7 +22232,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -22454,7 +22332,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -22660,7 +22537,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -22761,7 +22637,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -22967,7 +22842,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -23803,7 +23677,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -23904,7 +23777,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -24005,7 +23877,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -24106,7 +23977,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -24207,7 +24077,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -24308,7 +24177,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -24409,7 +24277,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -24510,7 +24377,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -24716,7 +24582,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -24817,7 +24682,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -25118,7 +24982,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -25209,7 +25072,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -25300,7 +25162,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -25391,7 +25252,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -25482,7 +25342,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -25573,7 +25432,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -25664,7 +25522,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -25755,7 +25612,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -25846,7 +25702,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -25937,7 +25792,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -26353,7 +26207,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -26454,7 +26307,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -27280,7 +27132,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -27376,7 +27227,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -27667,7 +27517,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -27763,7 +27612,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -27859,7 +27707,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -27955,7 +27802,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -28056,7 +27902,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -28157,7 +28002,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -28258,7 +28102,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -28359,7 +28202,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr"/>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -28460,7 +28302,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -28561,7 +28402,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -28662,7 +28502,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -28763,7 +28602,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -29679,7 +29517,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -29775,7 +29612,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -29871,7 +29707,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -29967,7 +29802,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -30063,7 +29897,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -30159,7 +29992,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -30255,7 +30087,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -30351,7 +30182,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -31652,7 +31482,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -31963,7 +31792,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -32064,7 +31892,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -32270,7 +32097,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -32686,7 +32512,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -32787,7 +32612,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -32888,7 +32712,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -33094,7 +32917,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -33300,7 +33122,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -33611,7 +33432,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -33712,7 +33532,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -33908,7 +33727,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -34004,7 +33822,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -34105,7 +33922,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -34311,7 +34127,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -35022,7 +34837,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -35123,7 +34937,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -35224,7 +35037,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -35320,7 +35132,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -35416,7 +35227,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -35512,7 +35322,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -35608,7 +35417,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -35704,7 +35512,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -36435,7 +36242,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -36536,7 +36342,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -36637,7 +36442,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -36738,7 +36542,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -36839,7 +36642,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -37045,7 +36847,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -37251,7 +37052,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -37457,7 +37257,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -37558,7 +37357,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -37764,7 +37562,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -37970,7 +37767,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U372" t="inlineStr"/>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
@@ -38596,7 +38392,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -38907,7 +38702,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U381" t="inlineStr"/>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
@@ -39318,7 +39112,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U385" t="inlineStr"/>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
@@ -39419,7 +39212,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -39520,7 +39312,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -39621,7 +39412,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -39722,7 +39512,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -40743,7 +40532,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -40844,7 +40632,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -40945,7 +40732,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -41046,7 +40832,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -41147,7 +40932,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -41248,7 +41032,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -41349,7 +41132,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -41450,7 +41232,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -41551,7 +41332,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -41652,7 +41432,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -42278,7 +42057,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -42379,7 +42157,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -42480,7 +42257,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -42581,7 +42357,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -42682,7 +42457,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -42783,7 +42557,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -42884,7 +42657,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -42985,7 +42757,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -43086,7 +42857,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -43187,7 +42957,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -43288,7 +43057,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -43389,7 +43157,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -43490,7 +43257,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -43591,7 +43357,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -43692,7 +43457,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -43893,7 +43657,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -44309,7 +44072,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -44410,7 +44172,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -44511,7 +44272,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -44612,7 +44372,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -44818,7 +44577,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -44919,7 +44677,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -45115,7 +44872,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -45311,7 +45067,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -45407,7 +45162,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -45503,7 +45257,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -45599,7 +45352,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -46095,7 +45847,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -46376,7 +46127,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -46687,7 +46437,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -46788,7 +46537,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -46889,7 +46637,6 @@
           <t>pipeline_extracted_in_validated_window</t>
         </is>
       </c>
-      <c r="U460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -47190,7 +46937,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -47291,7 +47037,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -47392,7 +47137,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -47488,7 +47232,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -47584,7 +47327,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -47680,7 +47422,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -48096,7 +47837,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -48197,7 +47937,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -48503,7 +48242,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -48599,7 +48337,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -48695,7 +48432,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -48796,7 +48532,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -48897,7 +48632,6 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -48998,7 +48732,465 @@
           <t>pipeline_extracted</t>
         </is>
       </c>
-      <c r="U481" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>07/24/2025</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>COUNTRY Mutual Insurance Company</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>19.0 Personal Auto</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>19.0000 Personal Auto Combinations</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>12.461%</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I482" t="n">
+        <v>14823</v>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>48935728</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>1697.200%</t>
+        </is>
+      </c>
+      <c r="L482" t="inlineStr">
+        <is>
+          <t>-69.600%</t>
+        </is>
+      </c>
+      <c r="M482" t="inlineStr">
+        <is>
+          <t>rate_change</t>
+        </is>
+      </c>
+      <c r="N482" t="inlineStr">
+        <is>
+          <t>CFPC-134508132</t>
+        </is>
+      </c>
+      <c r="O482" t="inlineStr">
+        <is>
+          <t>Filed</t>
+        </is>
+      </c>
+      <c r="P482" t="inlineStr">
+        <is>
+          <t>2025-05-01</t>
+        </is>
+      </c>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>output/pdfs/GA/134508132/filing_summary.pdf</t>
+        </is>
+      </c>
+      <c r="R482" t="inlineStr">
+        <is>
+          <t>pipeline_only</t>
+        </is>
+      </c>
+      <c r="S482" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="T482" t="inlineStr">
+        <is>
+          <t>pipeline_extracted_in_validated_window</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>09/21/2025</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>COUNTRY Mutual Insurance Company</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>19.0 Personal Auto</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>19.0000 Personal Auto Combinations</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>12.461%</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>3.614%</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>2319926</t>
+        </is>
+      </c>
+      <c r="I483" t="n">
+        <v>14823</v>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>64194422</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>1684.000%</t>
+        </is>
+      </c>
+      <c r="L483" t="inlineStr">
+        <is>
+          <t>-73.600%</t>
+        </is>
+      </c>
+      <c r="M483" t="inlineStr">
+        <is>
+          <t>rate_change</t>
+        </is>
+      </c>
+      <c r="N483" t="inlineStr">
+        <is>
+          <t>CFPC-134294144</t>
+        </is>
+      </c>
+      <c r="O483" t="inlineStr">
+        <is>
+          <t>Filed</t>
+        </is>
+      </c>
+      <c r="Q483" t="inlineStr">
+        <is>
+          <t>output/pdfs/GA/134294144/filing_summary.pdf</t>
+        </is>
+      </c>
+      <c r="R483" t="inlineStr">
+        <is>
+          <t>pipeline_only</t>
+        </is>
+      </c>
+      <c r="S483" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="T483" t="inlineStr">
+        <is>
+          <t>pipeline_extracted_in_validated_window</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>02/18/2024</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>COUNTRY Mutual Insurance Company</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>19.0 Personal Auto</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>19.0000 Personal Auto Combinations</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>39.590%</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>18.711%</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>3860999</t>
+        </is>
+      </c>
+      <c r="I484" t="n">
+        <v>5263</v>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>20635159</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>1384.500%</t>
+        </is>
+      </c>
+      <c r="L484" t="inlineStr">
+        <is>
+          <t>4.800%</t>
+        </is>
+      </c>
+      <c r="M484" t="inlineStr">
+        <is>
+          <t>rate_change</t>
+        </is>
+      </c>
+      <c r="N484" t="inlineStr">
+        <is>
+          <t>CFPC-133859077</t>
+        </is>
+      </c>
+      <c r="O484" t="inlineStr">
+        <is>
+          <t>Filed</t>
+        </is>
+      </c>
+      <c r="P484" t="inlineStr">
+        <is>
+          <t>2023-11-06</t>
+        </is>
+      </c>
+      <c r="Q484" t="inlineStr">
+        <is>
+          <t>output/pdfs/GA/133859077/filing_summary.pdf</t>
+        </is>
+      </c>
+      <c r="R484" t="inlineStr">
+        <is>
+          <t>pipeline_only</t>
+        </is>
+      </c>
+      <c r="S484" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="T484" t="inlineStr">
+        <is>
+          <t>pipeline_extracted</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>03/09/2025</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>COUNTRY Mutual Insurance Company</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>04.0 Homeowners</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>04.0000 Homeowners Sub-TOI Combinations</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="L485" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="M485" t="inlineStr">
+        <is>
+          <t>rate_change</t>
+        </is>
+      </c>
+      <c r="N485" t="inlineStr">
+        <is>
+          <t>CFPC-134290937</t>
+        </is>
+      </c>
+      <c r="O485" t="inlineStr">
+        <is>
+          <t>Acknowledged</t>
+        </is>
+      </c>
+      <c r="Q485" t="inlineStr">
+        <is>
+          <t>output/pdfs/GA/134290937/filing_summary.pdf</t>
+        </is>
+      </c>
+      <c r="R485" t="inlineStr">
+        <is>
+          <t>pipeline_only</t>
+        </is>
+      </c>
+      <c r="S485" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="T485" t="inlineStr">
+        <is>
+          <t>pipeline_extracted_in_validated_window</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>03/09/2025</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>COUNTRY Casualty Insurance Company</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>04.0 Homeowners</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>04.0000 Homeowners Sub-TOI Combinations</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="L486" t="inlineStr">
+        <is>
+          <t>0.000%</t>
+        </is>
+      </c>
+      <c r="M486" t="inlineStr">
+        <is>
+          <t>rate_change</t>
+        </is>
+      </c>
+      <c r="N486" t="inlineStr">
+        <is>
+          <t>CFPC-134290937</t>
+        </is>
+      </c>
+      <c r="O486" t="inlineStr">
+        <is>
+          <t>Acknowledged</t>
+        </is>
+      </c>
+      <c r="Q486" t="inlineStr">
+        <is>
+          <t>output/pdfs/GA/134290937/filing_summary.pdf</t>
+        </is>
+      </c>
+      <c r="R486" t="inlineStr">
+        <is>
+          <t>pipeline_only</t>
+        </is>
+      </c>
+      <c r="S486" t="inlineStr">
+        <is>
+          <t>original</t>
+        </is>
+      </c>
+      <c r="T486" t="inlineStr">
+        <is>
+          <t>pipeline_extracted_in_validated_window</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>